<commit_message>
added comments in all definitions
</commit_message>
<xml_diff>
--- a/extracted_links.xlsx
+++ b/extracted_links.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -440,186 +440,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>VIDEO: Pune Requires 5 Cyber Police Stations, Says BJP MLA Siddharth Shirole In Assembly</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://www.freepressjournal.in/pune/video-pune-requires-5-cyber-police-stations-says-bjp-mla-siddharth-shirole-in-assembly</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Pune Cyber Crime: MLA Siddharth Shirole Urges Approval for Five New Cyber Police Stations in Pune</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>https://www.thebridgechronicle.com/pune/pune-cyber-crime-mla-siddharth-shirole-demands-new-cyber-police-stations</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Merger of Cantonment Boards: Pune, Khadki to Join PMC, Aurangabad to Merge with Chhatrapati Sambhajinagar Municipal Corporation</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>https://www.punekarnews.in/merger-of-cantonment-boards-pune-khadki-to-join-pmc-aurangabad-to-merge-with-chhatrapati-sambhajinagar-municipal-corporation/</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Glass Found in Bun Maska at Pune's Iconic Goodluck Café Sparks Food Safety Concerns</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>https://www.thebridgechronicle.com/pune/glass-found-in-bun-maska-at-punes-goodluck-cafe-food-safety-concerns</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Bharat Bandh On July 9: What Will Be Closed &amp; What Will Be Open?</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>https://www.freepressjournal.in/business/bharat-bandh-on-july-9-railways-postal-services-banks-transport-services-to-be-closed</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Kanwar Yatra 2025: When Does It Begin? Date, Significance &amp; Rituals</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>https://www.freepressjournal.in/lifestyle/kanwar-yatra-2025-when-does-it-begin-date-significance-rituals</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>OpenAI To Launch AI-Powered Web Browser, Will Compete With Google Chrome, Perplexitys Comet</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>https://www.freepressjournal.in/tech/openai-to-launch-ai-powered-web-browser-will-compete-with-google-chrome-perplexitys-comet</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Nagaland State Lottery Result: July 10, 2025, 8 PM Live - Watch Streaming Of Winners List Of Dear Sandpiper</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>https://www.freepressjournal.in/india/nagaland-state-lottery-result-july-10-2025-8-pm-live-watch-streaming-of-winners-list-of-dear-sandpiper-sambad-night-thursday-weekly-draw</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Banks Should Free Frozen Accounts In Cyber Crimes After Submitting Police Certificates: Maha CM</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>https://menafn.com/1109785967/Banks-Should-Free-Frozen-Accounts-In-Cyber-Crimes-After-Submitting-Police-Certificates-Maha-CM</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>पुणे, खडकी, औरंगाबाद, देवळाली, अहमदनगर, कामटी कटकमंडळांचे महापालिकांमध्ये विलिनीकरण - मुख्यमंत्री देवेंद्र फडणवीस</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>https://mahasamvad.in/171950/</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Jansuraksha Bill: अखेर वादग्रस्त जनसुरक्षा विधेयक विधानसभेत सादर! मुख्यमंत्री म्हणाले, 12,000 हरकती अन्...</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>https://sarkarnama.esakal.com/mumbai/controversial-maharashtra-special-jansuraksha-bill-2024-finally-presented-by-cm-devendra-fadnavis-in-vidhan-sabha-aau85</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Monsoon Session : जन सुरक्षा विधेयक सभागृहात मांडताना मुख्यमंत्र्यांनी सांगितले, हे का महत्त्वाचे?</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>https://www.mymahanagar.com/maharashtra/monsoon-session-jansuraksha-act-maharashtra-cm-devendra-fadnavis-presented-in-assembly/</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>नक्षल, माओवादाचा कणा मोडणार - जनसुरक्षा विधेयक बहुमताने संमत; दुरूपयोग होणार नाही, मुख्यमंत्र्यांची ग्वाही</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>https://www.mahamtb.com/Encyc/2025/7/10/curbing-naxalism-and-maoism-however-it-will-not-be-misused.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>विधानसभा लक्षवेधी</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>https://mahasamvad.in/171905/</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>पुणे,खडकी,औरंगाबाद,देवळाली,अहिल्यानगर,कामटी कटकमंडळाचे विलिनीकरण मुख्यमंत्री देवेंद्र फडणवीस</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>https://awajmaharashtracha.news/bhingar-3/</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Link generation and news extraction merged successfully
</commit_message>
<xml_diff>
--- a/extracted_links.xlsx
+++ b/extracted_links.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -440,6 +440,438 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Maharashtra to set up state-level committee for effective leprosy eradication: Health Minister Prakash Abitkar</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.mid-day.com/mumbai/mumbai-news/article/maharashtra-to-set-up-state-level-committee-for-effective-leprosy-eradication-says-maharashtra-health-minister-prakash-abitkar-23584820</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Four new cancer hospitals to be set up in Maharashtra: Minister</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://www.lokmattimes.com/health/four-new-cancer-hospitals-to-be-set-up-in-maharashtra-minister-1/</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Reports of 14,000 Maha women with Cancer symptoms false: Minister | 'There have been a mismatch in figures' | Inshorts</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>https://inshorts.com/en/amp_news/reports-of-14-000-maha-women-with-cancer-symptoms-false--minister-1752313808066</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Mumbai Buzz: Top Headlines &amp; Latest News from the City That Never Sleeps</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>https://www.mid-day.com/mumbai/mumbai-news/photo/in-photos-maharashtra-to-form-leprosy-eradication-committee--106388</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>विस्कळीत झालेली, १०२ रुग्णवाहिका सेवा पूर्ववत ?</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>https://www.loksatta.com/mumbai/health-minister-prakash-abitkar-says-102-ambulance-service-restored-mumbai-print-news-ocd-94-5228346/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Mahayuti Controversy: कोल्हापुरात 10 आमदार असलेल्या महायुतीत वादाचा भडका; आबिटकरांनाच विरोध,भाजपनं घातला थेट मुद्द्यालाच हात</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://sarkarnama.esakal.com/maharashtra/paschim-maharashtra/mahayuti-dispute-over-kolhapur-district-committee-bjp-ncp-vs-prakash-abitkar-dk88-rg93</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>सरकारचा इशारा.. डाॅक्टर, कर्मचारी आरोग्य केंद्रात उपस्थित नसल्यास कारवाई! 334 खासगी रुग्णालयावर बंदी</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://marathi.oneindia.com/health/legislative-session-2025-action-will-be-taken-if-doctor-staff-is-not-present-in-phc-prakash-abitkar-032765.html?ref_source=OI-MR&amp;ref_medium=Home-Page&amp;ref_campaign=News-Cards</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>प्रकाश आबिटकर यांची माहिती, १०२ क्रमांक रुग्णवाहिका सेवा सुरळीत, कंत्राटी कर्मचाऱ्यांचे वेतन…</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://www.marathiebatmya.com/political/prakash-abitkar-informed-102-number-ambulance-service-on-regular/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Maharashtra : राज्यात 4 नव्या कर्करोग रुग्णालयांची निर्मिती करणार, आरोग्य मंत्र्यांची घोषणा</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://www.mymahanagar.com/maharashtra/maharashtra-4-new-cancer-hospital-will-developed-by-governement-says-health-minister-prakash-abitkar/</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>पन्हाळगडाचा जागतिक वारसास्थळात समावेश हा अभिमानाचा क्षण - पालकमंत्री आबिटकर</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>https://www.lokmat.com/kolhapur/inclusion-of-panhalgad-in-world-heritage-site-is-a-proud-moment-says-guardian-minister-prakash-abitkar-a-a746/</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ईएसआय रुग्णालयासाठी लवकरच नव्या सुविधा</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>https://deshdoot.com/new-facilities-soon-for-esi-hospital-health-minister-abitkar-assures-mla-seema-hire/</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>મહારાષ્ટ્રમાં એક જિલ્લામાં 14,000 મહિલાઓમાં મળ્યા કેન્સરના લક્ષણ, શું બોલ્યા સ્વાસ્થ્ય મંત્રી?</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>https://www.khabarchhe.com/national/maharashtra-over-14000-women-detected-with-cancer-like-symptoms-in-hingoli-health-minister-prakash-abitkar-tell-in-assembly/article-172633</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>प्रकाश आबिटकर यांच्याकडून गुरुजनांना विधानसभेची हवाई सैर</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>https://www.loksatta.com/kolhapur/kolhapur-minister-prakash-abitkar-takes-senior-citizens-on-air-trip-unique-guru-purnima-initiative-vsd-99-5224693/</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Kolhapur Politics : प्रकाश आबिटकरांना स्वकियांचेचं आव्हान, भाजप, अजित पवार गटाचा विरोध; जिल्हा नियोजन समितीवरून पडणार ठिणगी</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>https://www.esakal.com/paschim-maharashtra/kolhapur/prakash-abitkar-kolhapur-guardian-minister-faced-dissent-from-bjp-especially-shinde-aligned-factions-during-a-district-planning-committee-meeting-srs92</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Sangamner : महिलांच्या स्वतंत्र रुग्णालयाबाबत शासन सकारात्मक – ना. अबिटकर</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>https://deshdoot.com/women-hospital-health-minister-prakash-abitkar-statement-sangamner/</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Politics Kolhapur : आबिटकर, मुश्रीफ, कोरे, महाडिक, आवाडे, यड्रावकरांची डोकेदुखी वाढणार, अनेकांचा अपेक्षाभंग; सतेज पाटलांच्या भूमिकेकडे लक्ष</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>https://www.esakal.com/paschim-maharashtra/kolhapur/politics-kolhapur-headaches-of-prakash-abitkar-hasan-mushrif-vinay-kore-awade-yadravkar-will-increase-number-of-aspirants-what-is-the-role-of-satej-patil-srs92</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>मेगा रक्तदान शिबिराचे आयोजन करू नये; राज्य रक्त संक्रमण परिषदेच्या रक्तपेढ्यांना निर्देश</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>https://www.loksatta.com/mumbai/maharashtra-health-department-prakash-abitkar-limits-mega-blood-donation-camps-mumbai-print-news-rds-00-5227011/</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>वारसास्थळ यादीतील पन्हाळ्याचा समावेश अभिमानास्पद – आबिटकर</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>https://www.loksatta.com/kolhapur/inclusion-of-panhala-in-the-heritage-site-list-is-a-matter-of-pride-says-prakash-abitkar-ssb-93-5224775/</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>संगमनेरमध्ये महिलांसाठी स्वतंत्र रुग्णालय सुरू होणार, सार्वजनिक आरोग्यमंत्री प्रकाश अबिटकर यांची बैठकीत माहिती</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>https://ahmednagarlive24.com/ahilyanagar-news/a-separate-hospital-for-women-will-be-opened-in-sangamner-public-health-minister-prakash-abitkar-informed-in-a-meeting/</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Four new cancer hospitals to be set up in Maharashtra: Minister</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>https://www.socialnews.xyz/?p=6753712</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>महाराष्ट्राच्या हिंगोलीमध्ये १४ हजार महिलांमध्ये आढळला कर्करोग? येथे जाणून घ्या सत्य</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>https://newschecker.in/mr/fact-check-mr/14-5k-women-detected-cancer-in-hingoli/</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Four new cancer hospitals to be set up in Maharashtra: Minister</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>https://www.sakshipost.com/news/four-new-cancer-hospitals-be-set-maharashtra-minister-429363</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>छत्रपती शिवरायांचा इतिहास जगभर पोहोचणार, UNESCO यादीत पन्हाळगडाचा समावेश; पालकमंत्र्यांनी 'या' घटनेची करुन दिली आठवण</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>https://www.esakal.com/paschim-maharashtra/kolhapur/panhala-fort-unesco-world-heritage-site-shivaji-tourism-patrimony-prakash-abitkar-statement-bam92</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>People staying within 100m periphery of Panhala fort fear displacement</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>https://timesofindia.indiatimes.com/city/kolhapur/people-staying-within-100m-periphery-of-panhala-fort-fear-displacement/articleshow/122411210.cms</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Maha govt to set up committee for implementation of leprosy eradication</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>https://www.lokmattimes.com/national/maha-govt-to-set-up-committee-for-implementation-of-leprosy-eradication/</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Four new cancer hospitals to be set up in Maharashtra: Minister</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>https://www.socialnews.xyz/2025/07/15/four-new-cancer-hospitals-to-be-set-up-in-maharashtra-minister/</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>पावनखिंड तरुणांना ऊर्जा देणारी शिवमोहीम : पालकमंत्री आबिटकर -</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>https://livemarathi.in/shiv-mohim-energizing-the-youth-of-pawankhind-guardian-minister-abitkar/</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>‘नागरिकांसाठी समस्या, समाधान कक्ष’ स्थापन... -</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>https://livemarathi.in/problem-and-solution-room-for-citizens-established/</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Maha govt to set up committee for implementation of leprosy eradication</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>https://www.socialnews.xyz/2025/07/15/maha-govt-to-set-up-committee-for-implementation-of-leprosy-eradication/amp/</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Maharashtra Faces Cancer Crisis: Over 14500 Women in Hingoli Show ‘Cancer-Like’ Symptoms During Govt Health Screening</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>https://www.thehealthsite.com/news/maharashtra-faces-cancer-crisis-over-14500-women-in-hingoli-show-cancer-like-symptoms-during-govt-health-screening-1239129/</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Over 14,500 Women Detected With Cancer-Like Symptoms Post Screening In Maharashtra's Hingoli</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>https://www.msn.com/en-in/health/other/over-14500-women-detected-with-cancer-like-symptoms-post-screening-in-maharashtras-hingoli/ar-AA1Iqx6N</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Maharashtra Health Department to set up committee for effective leprosy eradication</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>https://www.thehindu.com/news/national/maharashtra/maharashtra-health-department-to-set-up-committee-for-effective-leprosy-eradication/article69815684.ece</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>कुष्ठरोग निर्मूलनाच्या प्रभावी अंमलबजावणीसाठी राज्यस्तरीय समिती स्थापन करणार -सार्वजनिक आरोग्यमंत्री प्रकाश आबिटकर</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>https://mahasamvad.in/172391/</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Monsoon Session : कुष्ठरोग निर्मूलन मोहिमेला नवे बळ; राज्यस्तरीय समिती स्थापन करण्याची आरोग्य मंत्र्यांची घोषणा</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>https://www.marathi.hindusthanpost.com/social/monsoon-session-new-strength-for-leprosy-eradication-campaign-health-minister-announces-formation-of-state-level-committee/</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>विधानसभा इतर कामकाज</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>https://mahasamvad.in/172498/</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>कुष्ठरोग निर्मूलनाच्या प्रभावी अंमलबजावणीसाठी राज्यस्तरीय समिती स्थापन करणार</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>https://dainikekmat.com/%E0%A4%95%E0%A5%81%E0%A4%B7%E0%A5%8D%E0%A4%A0%E0%A4%B0%E0%A5%8B%E0%A4%97-%E0%A4%A8%E0%A4%BF%E0%A4%B0%E0%A5%8D%E0%A4%AE%E0%A5%82%E0%A4%B2%E0%A4%A8%E0%A4%BE%E0%A4%9A%E0%A5%8D%E0%A4%AF%E0%A4%BE-%E0%A4%AA/109592/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>